<commit_message>
dev ver 0.3.55.5 1.修复了114514个bug
</commit_message>
<xml_diff>
--- a/other/RankTable.xlsx
+++ b/other/RankTable.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="77">
   <si>
     <t>9, 1, -3, -7</t>
   </si>
@@ -64,151 +64,172 @@
     <t>掉段</t>
   </si>
   <si>
+    <t>初级场均得pt</t>
+  </si>
+  <si>
+    <t>均失pt</t>
+  </si>
+  <si>
+    <t>均得系数(正负和)</t>
+  </si>
+  <si>
+    <t>高级场</t>
+  </si>
+  <si>
+    <t>四段及以上</t>
+  </si>
+  <si>
+    <t>无提示 无指针提示 错和 战术鸣牌</t>
+  </si>
+  <si>
+    <t>10级</t>
+  </si>
+  <si>
+    <t>无</t>
+  </si>
+  <si>
+    <t>MCRPL</t>
+  </si>
+  <si>
+    <t>达到salasasa七段、专业五段以上并实名</t>
+  </si>
+  <si>
+    <t>无提示 无指针提示 错和 战术鸣牌 禁止聊天 仅PC</t>
+  </si>
+  <si>
+    <t>9级</t>
+  </si>
+  <si>
+    <t>8级</t>
+  </si>
+  <si>
+    <t>计分系数 0.8均得pt，0.2均得pt，-0.3均失pt，-0.7均失pt</t>
+  </si>
+  <si>
+    <t>7级</t>
+  </si>
+  <si>
+    <t>6级</t>
+  </si>
+  <si>
+    <t>全庄均得系数</t>
+  </si>
+  <si>
+    <t>5级</t>
+  </si>
+  <si>
+    <t>初级场(全庄)</t>
+  </si>
+  <si>
+    <t>4级</t>
+  </si>
+  <si>
+    <t>中级场(全庄)</t>
+  </si>
+  <si>
+    <t>3级</t>
+  </si>
+  <si>
+    <t>有</t>
+  </si>
+  <si>
+    <t>高级场(全庄)</t>
+  </si>
+  <si>
+    <t>2级</t>
+  </si>
+  <si>
+    <t>MCRPL(全庄)</t>
+  </si>
+  <si>
+    <t>中级场均得pt</t>
+  </si>
+  <si>
+    <t>半庄均得系数</t>
+  </si>
+  <si>
+    <t>1级</t>
+  </si>
+  <si>
+    <t>初级场(半庄)</t>
+  </si>
+  <si>
+    <t>初段</t>
+  </si>
+  <si>
+    <t>中级场(半庄)</t>
+  </si>
+  <si>
+    <t>二段</t>
+  </si>
+  <si>
+    <t>高级场(半庄)</t>
+  </si>
+  <si>
+    <t>三段</t>
+  </si>
+  <si>
+    <t>MCRPL(半庄)</t>
+  </si>
+  <si>
+    <t>高级场均得pt</t>
+  </si>
+  <si>
+    <t>东风均得系数</t>
+  </si>
+  <si>
+    <t>四段</t>
+  </si>
+  <si>
+    <t>初级场(东风)</t>
+  </si>
+  <si>
+    <t>五段</t>
+  </si>
+  <si>
+    <t>中级场(东风)</t>
+  </si>
+  <si>
+    <t>六段</t>
+  </si>
+  <si>
+    <t>高级场(东风)</t>
+  </si>
+  <si>
+    <t>MCRPL均得pt</t>
+  </si>
+  <si>
+    <t>MCRPL(东风)</t>
+  </si>
+  <si>
+    <t>七段</t>
+  </si>
+  <si>
+    <t>八段</t>
+  </si>
+  <si>
+    <t>九段</t>
+  </si>
+  <si>
+    <t>十段</t>
+  </si>
+  <si>
+    <t>保留称号</t>
+  </si>
+  <si>
+    <t>天凤数据参考 平台的段位需要比天凤稍且严格</t>
+  </si>
+  <si>
     <t>均得pt</t>
   </si>
   <si>
-    <t>均失pt</t>
-  </si>
-  <si>
     <t>均得系数</t>
   </si>
   <si>
-    <t>高级场</t>
-  </si>
-  <si>
-    <t>四段及以上</t>
-  </si>
-  <si>
-    <t>无提示 无指针提示 错和 战术鸣牌</t>
-  </si>
-  <si>
-    <t>10级</t>
-  </si>
-  <si>
-    <t>无</t>
-  </si>
-  <si>
-    <t>MCRPL</t>
-  </si>
-  <si>
-    <t>达到salasasa七段、专业五段以上并实名</t>
-  </si>
-  <si>
-    <t>无提示 无指针提示 错和 战术鸣牌 禁止聊天 仅PC</t>
-  </si>
-  <si>
-    <t>9级</t>
-  </si>
-  <si>
-    <t>8级</t>
-  </si>
-  <si>
-    <t>计分系数 0.8均得pt，0.2均得pt，-0.3均失pt，-0.7均失pt</t>
-  </si>
-  <si>
-    <t>7级</t>
-  </si>
-  <si>
-    <t>6级</t>
-  </si>
-  <si>
-    <t>全庄均得系数</t>
-  </si>
-  <si>
-    <t>5级</t>
-  </si>
-  <si>
-    <t>初级场(全庄)</t>
-  </si>
-  <si>
-    <t>4级</t>
-  </si>
-  <si>
-    <t>中级场(全庄)</t>
-  </si>
-  <si>
-    <t>3级</t>
-  </si>
-  <si>
-    <t>有</t>
-  </si>
-  <si>
-    <t>高级场(全庄)</t>
-  </si>
-  <si>
-    <t>2级</t>
-  </si>
-  <si>
-    <t>MCRPL(全庄)</t>
-  </si>
-  <si>
-    <t>半庄均得系数</t>
-  </si>
-  <si>
-    <t>1级</t>
-  </si>
-  <si>
-    <t>初级场(半庄)</t>
-  </si>
-  <si>
-    <t>初段</t>
-  </si>
-  <si>
-    <t>中级场(半庄)</t>
-  </si>
-  <si>
-    <t>二段</t>
-  </si>
-  <si>
-    <t>高级场(半庄)</t>
-  </si>
-  <si>
-    <t>三段</t>
-  </si>
-  <si>
-    <t>MCRPL(半庄)</t>
-  </si>
-  <si>
-    <t>东风均得系数</t>
-  </si>
-  <si>
-    <t>四段</t>
-  </si>
-  <si>
-    <t>初级场(东风)</t>
-  </si>
-  <si>
-    <t>五段</t>
-  </si>
-  <si>
-    <t>中级场(东风)</t>
-  </si>
-  <si>
-    <t>六段</t>
-  </si>
-  <si>
-    <t>高级场(东风)</t>
-  </si>
-  <si>
-    <t>MCRPL(东风)</t>
-  </si>
-  <si>
-    <t>七段</t>
-  </si>
-  <si>
-    <t>八段</t>
-  </si>
-  <si>
-    <t>九段</t>
-  </si>
-  <si>
-    <t>十段</t>
-  </si>
-  <si>
-    <t>天凤数据参考 平台的段位需要比天凤稍且严格</t>
-  </si>
-  <si>
     <t>计分系数</t>
+  </si>
+  <si>
+    <t>场阶</t>
   </si>
   <si>
     <t>1位:0.8均得pt</t>
@@ -622,7 +643,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -634,6 +655,32 @@
       <left style="thin">
         <color theme="5"/>
       </left>
+      <right style="thin">
+        <color theme="5" tint="0.399975585192419"/>
+      </right>
+      <top style="thin">
+        <color theme="5"/>
+      </top>
+      <bottom style="thin">
+        <color theme="5" tint="0.399975585192419"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="5" tint="0.399975585192419"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="5"/>
+      </top>
+      <bottom style="thin">
+        <color theme="5" tint="0.399975585192419"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color theme="5" tint="0.399975585192419"/>
       </right>
@@ -782,6 +829,43 @@
     </border>
     <border>
       <left style="thin">
+        <color theme="5" tint="0.399975585192419"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="5" tint="0.399975585192419"/>
+      </top>
+      <bottom style="thin">
+        <color theme="5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="5" tint="0.399975585192419"/>
+      </top>
+      <bottom style="thin">
+        <color theme="5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="5"/>
+      </right>
+      <top style="thin">
+        <color theme="5" tint="0.399975585192419"/>
+      </top>
+      <bottom style="thin">
+        <color theme="5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
       <right style="thin">
@@ -904,7 +988,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="11">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="16">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
@@ -916,34 +1000,34 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="18">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="14">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="15">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="14">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="16">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="17">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="18">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="19">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="20">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="19">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="21">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="22">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="23">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="10" borderId="0">
@@ -1028,7 +1112,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1041,89 +1125,98 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1442,17 +1535,17 @@
   <dimension ref="B2:W54"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="6" max="6" width="11.875" customWidth="1"/>
-    <col min="8" max="8" width="10.625" customWidth="1"/>
+    <col min="6" max="6" width="13.25" customWidth="1"/>
+    <col min="8" max="8" width="15.625" customWidth="1"/>
     <col min="9" max="9" width="7.125" customWidth="1"/>
     <col min="10" max="10" width="12.25" customWidth="1"/>
-    <col min="14" max="14" width="5.5" style="18" customWidth="1"/>
+    <col min="14" max="14" width="5.5" style="20" customWidth="1"/>
     <col min="15" max="15" width="5.5" customWidth="1"/>
-    <col min="16" max="16" width="5.5" style="18" customWidth="1"/>
+    <col min="16" max="16" width="5.5" style="20" customWidth="1"/>
     <col min="17" max="17" width="5.5" customWidth="1"/>
-    <col min="18" max="18" width="5.5" style="18" customWidth="1"/>
+    <col min="18" max="18" width="5.5" style="20" customWidth="1"/>
     <col min="19" max="19" width="5.5" customWidth="1"/>
-    <col min="20" max="20" width="5.5" style="18" customWidth="1"/>
+    <col min="20" max="20" width="5.5" style="20" customWidth="1"/>
     <col min="21" max="21" width="5.5" customWidth="1"/>
     <col min="22" max="22" width="5.875" customWidth="1"/>
   </cols>
@@ -1461,1811 +1554,1810 @@
       <c r="F2" t="s">
         <v>0</v>
       </c>
-      <c r="J2" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="K2" s="19" t="s">
+      <c r="J2" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="K2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
-      <c r="P2" s="19" t="s">
+      <c r="L2" s="21"/>
+      <c r="M2" s="21"/>
+      <c r="N2" s="21"/>
+      <c r="O2" s="21"/>
+      <c r="P2" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="Q2" s="19"/>
-      <c r="R2" s="19"/>
-      <c r="S2" s="19"/>
-      <c r="T2" s="19"/>
-      <c r="U2" s="19"/>
-      <c r="V2" s="19"/>
-      <c r="W2" s="19"/>
+      <c r="Q2" s="21"/>
+      <c r="R2" s="21"/>
+      <c r="S2" s="21"/>
+      <c r="T2" s="21"/>
+      <c r="U2" s="21"/>
+      <c r="V2" s="21"/>
+      <c r="W2" s="21"/>
     </row>
     <row r="3" spans="2:23">
-      <c r="J3" s="19" t="s">
+      <c r="J3" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="19" t="s">
+      <c r="K3" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="19"/>
-      <c r="P3" s="19" t="s">
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="21"/>
+      <c r="P3" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="Q3" s="19"/>
-      <c r="R3" s="19"/>
-      <c r="S3" s="19"/>
-      <c r="T3" s="19"/>
-      <c r="U3" s="19"/>
-      <c r="V3" s="19"/>
-      <c r="W3" s="19"/>
+      <c r="Q3" s="21"/>
+      <c r="R3" s="21"/>
+      <c r="S3" s="21"/>
+      <c r="T3" s="21"/>
+      <c r="U3" s="21"/>
+      <c r="V3" s="21"/>
+      <c r="W3" s="21"/>
     </row>
     <row r="4" ht="18" customHeight="1" spans="2:23">
       <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="20" t="s">
+      <c r="G4" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H4" s="21" t="s">
+      <c r="H4" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="I4" s="21"/>
-      <c r="J4" s="19" t="s">
+      <c r="I4" s="23"/>
+      <c r="J4" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="19" t="s">
+      <c r="K4" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19" t="s">
+      <c r="L4" s="21"/>
+      <c r="M4" s="21"/>
+      <c r="N4" s="21"/>
+      <c r="O4" s="21"/>
+      <c r="P4" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="19"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="19"/>
-      <c r="U4" s="19"/>
-      <c r="V4" s="19"/>
-      <c r="W4" s="19"/>
+      <c r="Q4" s="21"/>
+      <c r="R4" s="21"/>
+      <c r="S4" s="21"/>
+      <c r="T4" s="21"/>
+      <c r="U4" s="21"/>
+      <c r="V4" s="21"/>
+      <c r="W4" s="21"/>
     </row>
     <row r="5" ht="18" customHeight="1" spans="2:23">
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="7">
         <v>0</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="7">
         <v>20</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="7">
         <f>J$10</f>
         <v>30</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="9">
         <v>0</v>
       </c>
-      <c r="H5" s="21">
+      <c r="H5" s="9">
         <f>(F5-G5)/F5</f>
         <v>1</v>
       </c>
-      <c r="I5" s="21"/>
-      <c r="J5" s="19" t="s">
+      <c r="I5" s="23"/>
+      <c r="J5" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="K5" s="22" t="s">
+      <c r="K5" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="22"/>
-      <c r="P5" s="19" t="s">
+      <c r="L5" s="24"/>
+      <c r="M5" s="24">
+        <v>1</v>
+      </c>
+      <c r="N5" s="24"/>
+      <c r="O5" s="24"/>
+      <c r="P5" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="Q5" s="19"/>
-      <c r="R5" s="19"/>
-      <c r="S5" s="19"/>
-      <c r="T5" s="19"/>
-      <c r="U5" s="19"/>
-      <c r="V5" s="19"/>
-      <c r="W5" s="19"/>
+      <c r="Q5" s="21"/>
+      <c r="R5" s="21"/>
+      <c r="S5" s="21"/>
+      <c r="T5" s="21"/>
+      <c r="U5" s="21"/>
+      <c r="V5" s="21"/>
+      <c r="W5" s="21"/>
     </row>
     <row r="6" ht="18" customHeight="1" spans="2:23">
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="9">
+      <c r="C6" s="11">
         <v>0</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="11">
         <v>20</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="11">
         <f t="shared" ref="F6:F13" si="0">J$10</f>
         <v>30</v>
       </c>
-      <c r="G6" s="13">
+      <c r="G6" s="15">
         <v>0</v>
       </c>
-      <c r="H6" s="21">
+      <c r="H6" s="15">
         <f t="shared" ref="H6:H26" si="1">(F6-G6)/F6</f>
         <v>1</v>
       </c>
-      <c r="J6" s="21"/>
-      <c r="K6" s="21"/>
-      <c r="L6" s="21"/>
-      <c r="M6" s="21"/>
-      <c r="N6" s="23"/>
-      <c r="O6" s="21"/>
-      <c r="P6" s="23"/>
-      <c r="Q6" s="21"/>
-      <c r="R6" s="23"/>
-      <c r="S6" s="21"/>
-      <c r="T6" s="23"/>
-      <c r="U6" s="21"/>
+      <c r="J6" s="23"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="23"/>
+      <c r="M6" s="23"/>
+      <c r="N6" s="25"/>
+      <c r="O6" s="23"/>
+      <c r="P6" s="25"/>
+      <c r="Q6" s="23"/>
+      <c r="R6" s="25"/>
+      <c r="S6" s="23"/>
+      <c r="T6" s="25"/>
+      <c r="U6" s="23"/>
     </row>
     <row r="7" ht="18" customHeight="1" spans="2:23">
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="7">
         <v>0</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="7">
         <v>20</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="7">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="9">
         <v>0</v>
       </c>
-      <c r="H7" s="21">
+      <c r="H7" s="9">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="J7" s="21"/>
-      <c r="K7" s="21"/>
-      <c r="L7" s="21"/>
-      <c r="M7" s="21"/>
-      <c r="N7" s="24" t="s">
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="O7" s="21"/>
-      <c r="P7" s="23"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="23"/>
-      <c r="S7" s="21"/>
-      <c r="T7" s="23"/>
-      <c r="U7" s="21"/>
+      <c r="O7" s="23"/>
+      <c r="P7" s="25"/>
+      <c r="Q7" s="23"/>
+      <c r="R7" s="25"/>
+      <c r="S7" s="23"/>
+      <c r="T7" s="25"/>
+      <c r="U7" s="23"/>
     </row>
     <row r="8" ht="18" customHeight="1" spans="2:23">
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C8" s="11">
         <v>0</v>
       </c>
-      <c r="D8" s="9">
+      <c r="D8" s="11">
         <v>20</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="9">
+      <c r="F8" s="11">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="G8" s="13">
+      <c r="G8" s="15">
         <v>0</v>
       </c>
-      <c r="H8" s="21">
+      <c r="H8" s="15">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="J8" s="21" t="s">
+      <c r="J8" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="K8" s="21"/>
-      <c r="L8" s="21"/>
-      <c r="M8" s="21"/>
-      <c r="N8" s="25"/>
-      <c r="O8" s="21"/>
-      <c r="P8" s="25"/>
-      <c r="Q8" s="21"/>
-      <c r="R8" s="25"/>
-      <c r="S8" s="21"/>
-      <c r="T8" s="25"/>
-      <c r="U8" s="21"/>
+      <c r="K8" s="23"/>
+      <c r="L8" s="23"/>
+      <c r="M8" s="23"/>
+      <c r="N8" s="27"/>
+      <c r="O8" s="23"/>
+      <c r="P8" s="27"/>
+      <c r="Q8" s="23"/>
+      <c r="R8" s="27"/>
+      <c r="S8" s="23"/>
+      <c r="T8" s="27"/>
+      <c r="U8" s="23"/>
     </row>
     <row r="9" ht="18" customHeight="1" spans="2:23">
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="7">
         <v>0</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="7">
         <v>40</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="7">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="9">
         <v>0</v>
       </c>
-      <c r="H9" s="21">
+      <c r="H9" s="9">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="J9" s="21" t="s">
+      <c r="J9" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="K9" s="21">
-        <v>1</v>
-      </c>
-      <c r="L9" s="21"/>
-      <c r="M9" s="21"/>
-      <c r="N9" s="23"/>
-      <c r="O9" s="21">
+      <c r="K9" s="23">
+        <v>1</v>
+      </c>
+      <c r="L9" s="23"/>
+      <c r="M9" s="23"/>
+      <c r="N9" s="25"/>
+      <c r="O9" s="23">
         <v>0.8</v>
       </c>
-      <c r="P9" s="23"/>
-      <c r="Q9" s="21">
+      <c r="P9" s="25"/>
+      <c r="Q9" s="23">
         <v>0.2</v>
       </c>
-      <c r="R9" s="23"/>
-      <c r="S9" s="21">
+      <c r="R9" s="25"/>
+      <c r="S9" s="23">
         <v>-0.3</v>
       </c>
-      <c r="T9" s="23"/>
-      <c r="U9" s="21">
+      <c r="T9" s="25"/>
+      <c r="U9" s="23">
         <v>-0.7</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" spans="2:23">
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="11">
         <v>0</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="11">
         <v>60</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="11">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="G10" s="13">
+      <c r="G10" s="15">
         <v>0</v>
       </c>
-      <c r="H10" s="21">
+      <c r="H10" s="15">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="J10" s="21">
+      <c r="J10" s="23">
         <v>30</v>
       </c>
-      <c r="K10" s="21"/>
-      <c r="L10" s="21" t="s">
+      <c r="K10" s="23"/>
+      <c r="L10" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="M10" s="21"/>
-      <c r="N10" s="23">
-        <v>1</v>
-      </c>
-      <c r="O10" s="21">
+      <c r="M10" s="23"/>
+      <c r="N10" s="25">
+        <v>1</v>
+      </c>
+      <c r="O10" s="23">
         <f>J10*O$9</f>
         <v>24</v>
       </c>
-      <c r="P10" s="23">
+      <c r="P10" s="25">
         <v>2</v>
       </c>
-      <c r="Q10" s="21">
+      <c r="Q10" s="23">
         <f>J10*Q$9</f>
         <v>6</v>
       </c>
-      <c r="R10" s="23">
+      <c r="R10" s="25">
         <v>3</v>
       </c>
-      <c r="S10" s="21">
+      <c r="S10" s="23">
         <f>J10*S$9</f>
         <v>-9</v>
       </c>
-      <c r="T10" s="23">
+      <c r="T10" s="25">
         <v>4</v>
       </c>
-      <c r="U10" s="21">
+      <c r="U10" s="23">
         <f>J10*U$9</f>
         <v>-21</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="2:23">
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="7">
         <v>0</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="7">
         <v>80</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="7">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="9">
         <v>0</v>
       </c>
-      <c r="H11" s="21">
+      <c r="H11" s="9">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="J11" s="21">
+      <c r="J11" s="23">
         <v>55</v>
       </c>
-      <c r="K11" s="21"/>
-      <c r="L11" s="21" t="s">
+      <c r="K11" s="23"/>
+      <c r="L11" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="M11" s="21"/>
-      <c r="N11" s="23">
-        <v>1</v>
-      </c>
-      <c r="O11" s="21">
+      <c r="M11" s="23"/>
+      <c r="N11" s="25">
+        <v>1</v>
+      </c>
+      <c r="O11" s="23">
         <f>J11*O$9</f>
         <v>44</v>
       </c>
-      <c r="P11" s="23">
+      <c r="P11" s="25">
         <v>2</v>
       </c>
-      <c r="Q11" s="21">
+      <c r="Q11" s="23">
         <f t="shared" ref="Q11:Q23" si="2">J11*Q$9</f>
         <v>11</v>
       </c>
-      <c r="R11" s="23">
+      <c r="R11" s="25">
         <v>3</v>
       </c>
-      <c r="S11" s="21">
+      <c r="S11" s="23">
         <f t="shared" ref="S11:S23" si="3">J11*S$9</f>
         <v>-16.5</v>
       </c>
-      <c r="T11" s="23">
+      <c r="T11" s="25">
         <v>4</v>
       </c>
-      <c r="U11" s="21">
+      <c r="U11" s="23">
         <f t="shared" ref="U11:U23" si="4">J11*U$9</f>
         <v>-38.5</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" spans="2:23">
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="11">
         <v>0</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="11">
         <v>100</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="F12" s="9">
+      <c r="F12" s="11">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="G12" s="13">
+      <c r="G12" s="15">
         <v>0</v>
       </c>
-      <c r="H12" s="21">
+      <c r="H12" s="15">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="J12" s="21">
+      <c r="J12" s="23">
         <v>95</v>
       </c>
-      <c r="K12" s="21"/>
-      <c r="L12" s="21" t="s">
+      <c r="K12" s="23"/>
+      <c r="L12" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="M12" s="21"/>
-      <c r="N12" s="23">
-        <v>1</v>
-      </c>
-      <c r="O12" s="21">
+      <c r="M12" s="23"/>
+      <c r="N12" s="25">
+        <v>1</v>
+      </c>
+      <c r="O12" s="23">
         <f>J12*O$9</f>
         <v>76</v>
       </c>
-      <c r="P12" s="23">
+      <c r="P12" s="25">
         <v>2</v>
       </c>
-      <c r="Q12" s="21">
+      <c r="Q12" s="23">
         <f t="shared" si="2"/>
         <v>19</v>
       </c>
-      <c r="R12" s="23">
+      <c r="R12" s="25">
         <v>3</v>
       </c>
-      <c r="S12" s="21">
+      <c r="S12" s="23">
         <f t="shared" si="3"/>
         <v>-28.5</v>
       </c>
-      <c r="T12" s="23">
+      <c r="T12" s="25">
         <v>4</v>
       </c>
-      <c r="U12" s="21">
+      <c r="U12" s="23">
         <f t="shared" si="4"/>
         <v>-66.5</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" spans="2:23">
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="15">
+      <c r="C13" s="17">
         <v>0</v>
       </c>
-      <c r="D13" s="15">
+      <c r="D13" s="17">
         <v>100</v>
       </c>
-      <c r="E13" s="15" t="s">
+      <c r="E13" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="F13" s="15">
+      <c r="F13" s="17">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="G13" s="26">
+      <c r="G13" s="28">
         <v>15</v>
       </c>
-      <c r="H13" s="21">
+      <c r="H13" s="28">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="J13" s="21">
+      <c r="J13" s="23">
         <v>135</v>
       </c>
-      <c r="K13" s="21"/>
-      <c r="L13" s="21" t="s">
+      <c r="K13" s="23"/>
+      <c r="L13" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="M13" s="21"/>
-      <c r="N13" s="23">
-        <v>1</v>
-      </c>
-      <c r="O13" s="21">
+      <c r="M13" s="23"/>
+      <c r="N13" s="25">
+        <v>1</v>
+      </c>
+      <c r="O13" s="23">
         <f t="shared" ref="O13:O23" si="5">J13*O$9</f>
         <v>108</v>
       </c>
-      <c r="P13" s="23">
+      <c r="P13" s="25">
         <v>2</v>
       </c>
-      <c r="Q13" s="21">
+      <c r="Q13" s="23">
         <f t="shared" si="2"/>
         <v>27</v>
       </c>
-      <c r="R13" s="23">
+      <c r="R13" s="25">
         <v>3</v>
       </c>
-      <c r="S13" s="21">
+      <c r="S13" s="23">
         <f t="shared" si="3"/>
         <v>-40.5</v>
       </c>
-      <c r="T13" s="23">
+      <c r="T13" s="25">
         <v>4</v>
       </c>
-      <c r="U13" s="21">
+      <c r="U13" s="23">
         <f t="shared" si="4"/>
         <v>-94.5</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1" spans="2:23">
-      <c r="B14" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="3" t="s">
+      <c r="B14" s="2"/>
+      <c r="C14" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F14" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G14" s="20" t="s">
+      <c r="F14" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H14" s="21"/>
-      <c r="J14" s="21" t="s">
-        <v>37</v>
-      </c>
-      <c r="K14" s="21">
+      <c r="H14" s="22"/>
+      <c r="J14" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="K14" s="23">
         <v>0.7</v>
       </c>
-      <c r="L14" s="21"/>
-      <c r="M14" s="21"/>
-      <c r="N14" s="23"/>
-      <c r="O14" s="21"/>
-      <c r="P14" s="23"/>
-      <c r="Q14" s="21"/>
-      <c r="R14" s="23"/>
-      <c r="S14" s="21"/>
-      <c r="T14" s="23"/>
-      <c r="U14" s="21"/>
+      <c r="L14" s="23"/>
+      <c r="M14" s="23"/>
+      <c r="N14" s="25"/>
+      <c r="O14" s="23"/>
+      <c r="P14" s="25"/>
+      <c r="Q14" s="23"/>
+      <c r="R14" s="25"/>
+      <c r="S14" s="23"/>
+      <c r="T14" s="25"/>
+      <c r="U14" s="23"/>
     </row>
     <row r="15" ht="18" customHeight="1" spans="2:23">
-      <c r="B15" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C15" s="5">
+      <c r="B15" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="7">
         <v>0</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="7">
         <v>100</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="7">
         <v>55</v>
       </c>
-      <c r="G15" s="7">
+      <c r="G15" s="9">
         <v>35</v>
       </c>
-      <c r="H15" s="21">
+      <c r="H15" s="9">
         <f t="shared" si="1"/>
         <v>0.363636363636364</v>
       </c>
-      <c r="J15" s="21">
+      <c r="J15" s="23">
         <f>J10*K$14</f>
         <v>21</v>
       </c>
-      <c r="K15" s="21"/>
-      <c r="L15" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="M15" s="21"/>
-      <c r="N15" s="23">
-        <v>1</v>
-      </c>
-      <c r="O15" s="21">
+      <c r="K15" s="23"/>
+      <c r="L15" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="M15" s="23"/>
+      <c r="N15" s="25">
+        <v>1</v>
+      </c>
+      <c r="O15" s="23">
         <f t="shared" si="5"/>
         <v>16.8</v>
       </c>
-      <c r="P15" s="23">
+      <c r="P15" s="25">
         <v>2</v>
       </c>
-      <c r="Q15" s="21">
+      <c r="Q15" s="23">
         <f t="shared" si="2"/>
         <v>4.2</v>
       </c>
-      <c r="R15" s="23">
+      <c r="R15" s="25">
         <v>3</v>
       </c>
-      <c r="S15" s="21">
+      <c r="S15" s="23">
         <f t="shared" si="3"/>
         <v>-6.3</v>
       </c>
-      <c r="T15" s="23">
+      <c r="T15" s="25">
         <v>4</v>
       </c>
-      <c r="U15" s="21">
+      <c r="U15" s="23">
         <f t="shared" si="4"/>
         <v>-14.7</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1" spans="2:23">
-      <c r="B16" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" s="9">
+      <c r="B16" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="11">
         <f>D16*0.5</f>
         <v>200</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="11">
         <v>400</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F16" s="11">
         <v>55</v>
       </c>
-      <c r="G16" s="13">
+      <c r="G16" s="15">
         <v>45</v>
       </c>
-      <c r="H16" s="21">
+      <c r="H16" s="15">
         <f t="shared" si="1"/>
         <v>0.181818181818182</v>
       </c>
-      <c r="J16" s="21">
+      <c r="J16" s="23">
         <f>J11*K$14</f>
         <v>38.5</v>
       </c>
-      <c r="K16" s="21"/>
-      <c r="L16" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="M16" s="21"/>
-      <c r="N16" s="23">
-        <v>1</v>
-      </c>
-      <c r="O16" s="21">
+      <c r="K16" s="23"/>
+      <c r="L16" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="M16" s="23"/>
+      <c r="N16" s="25">
+        <v>1</v>
+      </c>
+      <c r="O16" s="23">
         <f t="shared" si="5"/>
         <v>30.8</v>
       </c>
-      <c r="P16" s="23">
+      <c r="P16" s="25">
         <v>2</v>
       </c>
-      <c r="Q16" s="21">
+      <c r="Q16" s="23">
         <f t="shared" si="2"/>
         <v>7.7</v>
       </c>
-      <c r="R16" s="23">
+      <c r="R16" s="25">
         <v>3</v>
       </c>
-      <c r="S16" s="21">
+      <c r="S16" s="23">
         <f t="shared" si="3"/>
         <v>-11.55</v>
       </c>
-      <c r="T16" s="23">
+      <c r="T16" s="25">
         <v>4</v>
       </c>
-      <c r="U16" s="21">
+      <c r="U16" s="23">
         <f t="shared" si="4"/>
         <v>-26.95</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" spans="2:21">
-      <c r="B17" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C17" s="5">
+      <c r="B17" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17" s="7">
         <f t="shared" ref="C17:C26" si="6">D17*0.5</f>
         <v>400</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="7">
         <v>800</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="F17" s="5">
+      <c r="F17" s="7">
         <v>55</v>
       </c>
-      <c r="G17" s="7">
+      <c r="G17" s="9">
         <v>55</v>
       </c>
-      <c r="H17" s="21">
+      <c r="H17" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J17" s="21">
+      <c r="J17" s="23">
         <f>J12*K$14</f>
         <v>66.5</v>
       </c>
-      <c r="K17" s="21"/>
-      <c r="L17" s="21" t="s">
-        <v>43</v>
-      </c>
-      <c r="M17" s="21"/>
-      <c r="N17" s="23">
-        <v>1</v>
-      </c>
-      <c r="O17" s="21">
+      <c r="K17" s="23"/>
+      <c r="L17" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="M17" s="23"/>
+      <c r="N17" s="25">
+        <v>1</v>
+      </c>
+      <c r="O17" s="23">
         <f t="shared" si="5"/>
         <v>53.2</v>
       </c>
-      <c r="P17" s="23">
+      <c r="P17" s="25">
         <v>2</v>
       </c>
-      <c r="Q17" s="21">
+      <c r="Q17" s="23">
         <f t="shared" si="2"/>
         <v>13.3</v>
       </c>
-      <c r="R17" s="23">
+      <c r="R17" s="25">
         <v>3</v>
       </c>
-      <c r="S17" s="21">
+      <c r="S17" s="23">
         <f t="shared" si="3"/>
         <v>-19.95</v>
       </c>
-      <c r="T17" s="23">
+      <c r="T17" s="25">
         <v>4</v>
       </c>
-      <c r="U17" s="21">
+      <c r="U17" s="23">
         <f t="shared" si="4"/>
         <v>-46.55</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" spans="2:21">
-      <c r="B18" s="27" t="s">
-        <v>44</v>
-      </c>
-      <c r="C18" s="28">
+      <c r="B18" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="30">
         <f t="shared" si="6"/>
         <v>600</v>
       </c>
-      <c r="D18" s="28">
+      <c r="D18" s="30">
         <v>1200</v>
       </c>
-      <c r="E18" s="28" t="s">
+      <c r="E18" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="F18" s="28">
+      <c r="F18" s="30">
         <v>55</v>
       </c>
-      <c r="G18" s="29">
+      <c r="G18" s="31">
         <v>65</v>
       </c>
-      <c r="H18" s="21">
+      <c r="H18" s="31">
         <f t="shared" si="1"/>
         <v>-0.181818181818182</v>
       </c>
-      <c r="J18" s="21">
+      <c r="J18" s="23">
         <f>J13*K$14</f>
         <v>94.5</v>
       </c>
-      <c r="K18" s="21"/>
-      <c r="L18" s="21" t="s">
-        <v>45</v>
-      </c>
-      <c r="M18" s="21"/>
-      <c r="N18" s="23">
-        <v>1</v>
-      </c>
-      <c r="O18" s="21">
+      <c r="K18" s="23"/>
+      <c r="L18" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="M18" s="23"/>
+      <c r="N18" s="25">
+        <v>1</v>
+      </c>
+      <c r="O18" s="23">
         <f t="shared" si="5"/>
         <v>75.6</v>
       </c>
-      <c r="P18" s="23">
+      <c r="P18" s="25">
         <v>2</v>
       </c>
-      <c r="Q18" s="21">
+      <c r="Q18" s="23">
         <f t="shared" si="2"/>
         <v>18.9</v>
       </c>
-      <c r="R18" s="23">
+      <c r="R18" s="25">
         <v>3</v>
       </c>
-      <c r="S18" s="21">
+      <c r="S18" s="23">
         <f t="shared" si="3"/>
         <v>-28.35</v>
       </c>
-      <c r="T18" s="23">
+      <c r="T18" s="25">
         <v>4</v>
       </c>
-      <c r="U18" s="21">
+      <c r="U18" s="23">
         <f t="shared" si="4"/>
         <v>-66.15</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1" spans="2:21">
-      <c r="B19" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C19" s="3" t="s">
+      <c r="B19" s="2"/>
+      <c r="C19" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F19" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G19" s="20" t="s">
+      <c r="F19" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G19" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H19" s="21"/>
-      <c r="J19" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="K19" s="21">
+      <c r="H19" s="22"/>
+      <c r="J19" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="K19" s="23">
         <v>0.49</v>
       </c>
-      <c r="L19" s="21"/>
-      <c r="M19" s="21"/>
-      <c r="N19" s="23"/>
-      <c r="O19" s="21"/>
-      <c r="P19" s="23"/>
-      <c r="Q19" s="21"/>
-      <c r="R19" s="23"/>
-      <c r="S19" s="21"/>
-      <c r="T19" s="23"/>
-      <c r="U19" s="21"/>
+      <c r="L19" s="23"/>
+      <c r="M19" s="23"/>
+      <c r="N19" s="25"/>
+      <c r="O19" s="23"/>
+      <c r="P19" s="25"/>
+      <c r="Q19" s="23"/>
+      <c r="R19" s="25"/>
+      <c r="S19" s="23"/>
+      <c r="T19" s="25"/>
+      <c r="U19" s="23"/>
     </row>
     <row r="20" ht="18" customHeight="1" spans="2:21">
-      <c r="B20" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C20" s="5">
+      <c r="B20" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="7">
         <f t="shared" si="6"/>
         <v>800</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D20" s="7">
         <v>1600</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E20" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="F20" s="5">
+      <c r="F20" s="7">
         <v>95</v>
       </c>
-      <c r="G20" s="7">
+      <c r="G20" s="9">
         <v>95</v>
       </c>
-      <c r="H20" s="21">
+      <c r="H20" s="9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J20" s="21">
+      <c r="J20" s="23">
         <f>J10*K$19</f>
         <v>14.7</v>
       </c>
-      <c r="K20" s="21"/>
-      <c r="L20" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="M20" s="21"/>
-      <c r="N20" s="23">
-        <v>1</v>
-      </c>
-      <c r="O20" s="21">
+      <c r="K20" s="23"/>
+      <c r="L20" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="M20" s="23"/>
+      <c r="N20" s="25">
+        <v>1</v>
+      </c>
+      <c r="O20" s="23">
         <f t="shared" si="5"/>
         <v>11.76</v>
       </c>
-      <c r="P20" s="23">
+      <c r="P20" s="25">
         <v>2</v>
       </c>
-      <c r="Q20" s="21">
+      <c r="Q20" s="23">
         <f t="shared" si="2"/>
         <v>2.94</v>
       </c>
-      <c r="R20" s="23">
+      <c r="R20" s="25">
         <v>3</v>
       </c>
-      <c r="S20" s="21">
+      <c r="S20" s="23">
         <f t="shared" si="3"/>
         <v>-4.41</v>
       </c>
-      <c r="T20" s="23">
+      <c r="T20" s="25">
         <v>4</v>
       </c>
-      <c r="U20" s="21">
+      <c r="U20" s="23">
         <f t="shared" si="4"/>
         <v>-10.29</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1" spans="2:21">
-      <c r="B21" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C21" s="9">
+      <c r="B21" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C21" s="11">
         <f t="shared" si="6"/>
         <v>1000</v>
       </c>
-      <c r="D21" s="9">
+      <c r="D21" s="11">
         <v>2000</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="F21" s="9">
+      <c r="F21" s="11">
         <v>95</v>
       </c>
-      <c r="G21" s="13">
+      <c r="G21" s="15">
         <v>105</v>
       </c>
-      <c r="H21" s="21">
+      <c r="H21" s="15">
         <f t="shared" si="1"/>
         <v>-0.105263157894737</v>
       </c>
-      <c r="J21" s="21">
+      <c r="J21" s="23">
         <f>J11*K$19</f>
         <v>26.95</v>
       </c>
-      <c r="K21" s="21"/>
-      <c r="L21" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="M21" s="21"/>
-      <c r="N21" s="23">
-        <v>1</v>
-      </c>
-      <c r="O21" s="21">
+      <c r="K21" s="23"/>
+      <c r="L21" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="M21" s="23"/>
+      <c r="N21" s="25">
+        <v>1</v>
+      </c>
+      <c r="O21" s="23">
         <f t="shared" si="5"/>
         <v>21.56</v>
       </c>
-      <c r="P21" s="23">
+      <c r="P21" s="25">
         <v>2</v>
       </c>
-      <c r="Q21" s="21">
+      <c r="Q21" s="23">
         <f t="shared" si="2"/>
         <v>5.39</v>
       </c>
-      <c r="R21" s="23">
+      <c r="R21" s="25">
         <v>3</v>
       </c>
-      <c r="S21" s="21">
+      <c r="S21" s="23">
         <f t="shared" si="3"/>
         <v>-8.085</v>
       </c>
-      <c r="T21" s="23">
+      <c r="T21" s="25">
         <v>4</v>
       </c>
-      <c r="U21" s="21">
+      <c r="U21" s="23">
         <f t="shared" si="4"/>
         <v>-18.865</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1" spans="2:21">
-      <c r="B22" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="C22" s="15">
+      <c r="B22" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="17">
         <f t="shared" si="6"/>
         <v>1200</v>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="17">
         <v>2400</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="E22" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="F22" s="15">
+      <c r="F22" s="17">
         <v>95</v>
       </c>
-      <c r="G22" s="26">
+      <c r="G22" s="28">
         <v>120</v>
       </c>
-      <c r="H22" s="21">
+      <c r="H22" s="28">
         <f t="shared" si="1"/>
         <v>-0.263157894736842</v>
       </c>
-      <c r="J22" s="21">
+      <c r="J22" s="23">
         <f>J12*K$19</f>
         <v>46.55</v>
       </c>
-      <c r="K22" s="21"/>
-      <c r="L22" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="M22" s="21"/>
-      <c r="N22" s="23">
-        <v>1</v>
-      </c>
-      <c r="O22" s="21">
+      <c r="K22" s="23"/>
+      <c r="L22" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="M22" s="23"/>
+      <c r="N22" s="25">
+        <v>1</v>
+      </c>
+      <c r="O22" s="23">
         <f t="shared" si="5"/>
         <v>37.24</v>
       </c>
-      <c r="P22" s="23">
+      <c r="P22" s="25">
         <v>2</v>
       </c>
-      <c r="Q22" s="21">
+      <c r="Q22" s="23">
         <f t="shared" si="2"/>
         <v>9.31</v>
       </c>
-      <c r="R22" s="23">
+      <c r="R22" s="25">
         <v>3</v>
       </c>
-      <c r="S22" s="21">
+      <c r="S22" s="23">
         <f t="shared" si="3"/>
         <v>-13.965</v>
       </c>
-      <c r="T22" s="23">
+      <c r="T22" s="25">
         <v>4</v>
       </c>
-      <c r="U22" s="21">
+      <c r="U22" s="23">
         <f t="shared" si="4"/>
         <v>-32.585</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1" spans="2:21">
-      <c r="B23" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C23" s="3" t="s">
+      <c r="B23" s="2"/>
+      <c r="C23" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E23" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F23" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G23" s="20" t="s">
+      <c r="F23" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="G23" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H23" s="21"/>
-      <c r="J23" s="21">
+      <c r="H23" s="22"/>
+      <c r="J23" s="23">
         <f>J13*K$19</f>
         <v>66.15</v>
       </c>
-      <c r="K23" s="21"/>
-      <c r="L23" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="M23" s="21"/>
-      <c r="N23" s="23">
-        <v>1</v>
-      </c>
-      <c r="O23" s="21">
+      <c r="K23" s="23"/>
+      <c r="L23" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="M23" s="23"/>
+      <c r="N23" s="25">
+        <v>1</v>
+      </c>
+      <c r="O23" s="23">
         <f t="shared" si="5"/>
         <v>52.92</v>
       </c>
-      <c r="P23" s="23">
+      <c r="P23" s="25">
         <v>2</v>
       </c>
-      <c r="Q23" s="21">
+      <c r="Q23" s="23">
         <f t="shared" si="2"/>
         <v>13.23</v>
       </c>
-      <c r="R23" s="23">
+      <c r="R23" s="25">
         <v>3</v>
       </c>
-      <c r="S23" s="21">
+      <c r="S23" s="23">
         <f t="shared" si="3"/>
         <v>-19.845</v>
       </c>
-      <c r="T23" s="23">
+      <c r="T23" s="25">
         <v>4</v>
       </c>
-      <c r="U23" s="21">
+      <c r="U23" s="23">
         <f t="shared" si="4"/>
         <v>-46.305</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1" spans="2:21">
-      <c r="B24" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C24" s="5">
+      <c r="B24" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C24" s="7">
         <f t="shared" si="6"/>
         <v>1400</v>
       </c>
-      <c r="D24" s="5">
+      <c r="D24" s="7">
         <v>2800</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E24" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="F24" s="5">
+      <c r="F24" s="7">
         <v>135</v>
       </c>
-      <c r="G24" s="7">
+      <c r="G24" s="9">
         <v>150</v>
       </c>
-      <c r="H24" s="21">
+      <c r="H24" s="9">
         <f t="shared" si="1"/>
         <v>-0.111111111111111</v>
       </c>
-      <c r="J24" s="21"/>
-      <c r="K24" s="21"/>
-      <c r="L24" s="21"/>
-      <c r="M24" s="21"/>
-      <c r="N24" s="23"/>
-      <c r="O24" s="21"/>
-      <c r="P24" s="23"/>
-      <c r="Q24" s="21"/>
-      <c r="R24" s="23"/>
-      <c r="S24" s="21"/>
-      <c r="T24" s="23"/>
-      <c r="U24" s="21"/>
+      <c r="J24" s="23"/>
+      <c r="K24" s="23"/>
+      <c r="L24" s="23"/>
+      <c r="M24" s="23"/>
+      <c r="N24" s="25"/>
+      <c r="O24" s="23"/>
+      <c r="P24" s="25"/>
+      <c r="Q24" s="23"/>
+      <c r="R24" s="25"/>
+      <c r="S24" s="23"/>
+      <c r="T24" s="25"/>
+      <c r="U24" s="23"/>
     </row>
     <row r="25" ht="18" customHeight="1" spans="2:21">
-      <c r="B25" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="C25" s="9">
+      <c r="B25" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C25" s="11">
         <f t="shared" si="6"/>
         <v>1600</v>
       </c>
-      <c r="D25" s="9">
+      <c r="D25" s="11">
         <v>3200</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="F25" s="9">
+      <c r="F25" s="11">
         <v>135</v>
       </c>
-      <c r="G25" s="13">
+      <c r="G25" s="15">
         <v>175</v>
       </c>
-      <c r="H25" s="21">
+      <c r="H25" s="15">
         <f t="shared" si="1"/>
         <v>-0.296296296296296</v>
       </c>
-      <c r="J25" s="21"/>
-      <c r="K25" s="21"/>
-      <c r="L25" s="21"/>
-      <c r="M25" s="21"/>
-      <c r="N25" s="23"/>
-      <c r="O25" s="21"/>
-      <c r="P25" s="23"/>
-      <c r="Q25" s="21"/>
-      <c r="R25" s="23"/>
-      <c r="S25" s="21"/>
-      <c r="T25" s="23"/>
-      <c r="U25" s="21"/>
+      <c r="J25" s="23"/>
+      <c r="K25" s="23"/>
+      <c r="L25" s="23"/>
+      <c r="M25" s="23"/>
+      <c r="N25" s="25"/>
+      <c r="O25" s="23"/>
+      <c r="P25" s="25"/>
+      <c r="Q25" s="23"/>
+      <c r="R25" s="25"/>
+      <c r="S25" s="23"/>
+      <c r="T25" s="25"/>
+      <c r="U25" s="23"/>
     </row>
     <row r="26" ht="18" customHeight="1" spans="2:21">
-      <c r="B26" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C26" s="5">
+      <c r="B26" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" s="7">
         <f t="shared" si="6"/>
         <v>2000</v>
       </c>
-      <c r="D26" s="5">
+      <c r="D26" s="7">
         <v>4000</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="E26" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="F26" s="5">
+      <c r="F26" s="7">
         <v>135</v>
       </c>
-      <c r="G26" s="7">
+      <c r="G26" s="9">
         <v>190</v>
       </c>
-      <c r="H26" s="21">
+      <c r="H26" s="9">
         <f t="shared" si="1"/>
         <v>-0.407407407407407</v>
       </c>
-      <c r="J26" s="21"/>
-      <c r="K26" s="21"/>
-      <c r="L26" s="21"/>
-      <c r="M26" s="21"/>
-      <c r="N26" s="23"/>
-      <c r="O26" s="21"/>
-      <c r="P26" s="23"/>
-      <c r="Q26" s="21"/>
-      <c r="R26" s="23"/>
-      <c r="S26" s="21"/>
-      <c r="T26" s="23"/>
-      <c r="U26" s="21"/>
+      <c r="J26" s="23"/>
+      <c r="K26" s="23"/>
+      <c r="L26" s="23"/>
+      <c r="M26" s="23"/>
+      <c r="N26" s="25"/>
+      <c r="O26" s="23"/>
+      <c r="P26" s="25"/>
+      <c r="Q26" s="23"/>
+      <c r="R26" s="25"/>
+      <c r="S26" s="23"/>
+      <c r="T26" s="25"/>
+      <c r="U26" s="23"/>
     </row>
     <row r="27" ht="18" customHeight="1" spans="2:21">
-      <c r="B27" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="C27" s="30"/>
-      <c r="D27" s="28"/>
-      <c r="E27" s="30"/>
-      <c r="F27" s="30"/>
-      <c r="G27" s="31"/>
-      <c r="J27" s="21"/>
-      <c r="K27" s="21"/>
-      <c r="L27" s="21"/>
-      <c r="M27" s="21"/>
-      <c r="N27" s="23"/>
-      <c r="O27" s="21"/>
-      <c r="P27" s="23"/>
-      <c r="Q27" s="21"/>
-      <c r="R27" s="23"/>
-      <c r="S27" s="21"/>
-      <c r="T27" s="23"/>
-      <c r="U27" s="21"/>
+      <c r="B27" s="29" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="33"/>
+      <c r="H27" s="34"/>
+      <c r="J27" s="23"/>
+      <c r="K27" s="23"/>
+      <c r="L27" s="23"/>
+      <c r="M27" s="23"/>
+      <c r="N27" s="25"/>
+      <c r="O27" s="23"/>
+      <c r="P27" s="25"/>
+      <c r="Q27" s="23"/>
+      <c r="R27" s="25"/>
+      <c r="S27" s="23"/>
+      <c r="T27" s="25"/>
+      <c r="U27" s="23"/>
     </row>
     <row r="28" spans="2:21">
-      <c r="D28" s="21"/>
-      <c r="J28" s="21"/>
-      <c r="K28" s="21"/>
-      <c r="L28" s="21"/>
-      <c r="M28" s="21"/>
-      <c r="N28" s="23"/>
-      <c r="O28" s="21"/>
-      <c r="P28" s="23"/>
-      <c r="Q28" s="21"/>
-      <c r="R28" s="23"/>
-      <c r="S28" s="21"/>
-      <c r="T28" s="23"/>
-      <c r="U28" s="21"/>
+      <c r="D28" s="23"/>
+      <c r="J28" s="23"/>
+      <c r="K28" s="23"/>
+      <c r="L28" s="23"/>
+      <c r="M28" s="23"/>
+      <c r="N28" s="25"/>
+      <c r="O28" s="23"/>
+      <c r="P28" s="25"/>
+      <c r="Q28" s="23"/>
+      <c r="R28" s="25"/>
+      <c r="S28" s="23"/>
+      <c r="T28" s="25"/>
+      <c r="U28" s="23"/>
     </row>
     <row r="30" spans="2:21">
-      <c r="B30" s="32" t="s">
-        <v>58</v>
-      </c>
-      <c r="C30" s="32"/>
-      <c r="D30" s="32"/>
-      <c r="E30" s="32"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
-      <c r="H30" s="32"/>
+      <c r="B30" s="35" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" s="35"/>
+      <c r="D30" s="35"/>
+      <c r="E30" s="35"/>
+      <c r="F30" s="35"/>
+      <c r="G30" s="35"/>
+      <c r="H30" s="35"/>
     </row>
     <row r="31" spans="2:21">
-      <c r="B31" s="21"/>
-      <c r="C31" s="21" t="s">
+      <c r="B31" s="23"/>
+      <c r="C31" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="D31" s="21" t="s">
+      <c r="D31" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="E31" s="21" t="s">
+      <c r="E31" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="F31" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="G31" s="21" t="s">
+      <c r="F31" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="G31" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="H31" s="21" t="s">
-        <v>13</v>
+      <c r="H31" s="23" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="32" spans="2:21">
-      <c r="B32" s="21" t="s">
+      <c r="B32" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="C32" s="21">
+      <c r="C32" s="23">
         <v>0</v>
       </c>
-      <c r="D32" s="21">
+      <c r="D32" s="23">
         <v>20</v>
       </c>
-      <c r="E32" s="21" t="s">
+      <c r="E32" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="F32" s="21">
+      <c r="F32" s="23">
         <v>45</v>
       </c>
-      <c r="G32" s="21">
+      <c r="G32" s="23">
         <v>0</v>
       </c>
-      <c r="H32" s="21">
+      <c r="H32" s="23">
         <f t="shared" ref="H32:H40" si="7">(F32-G32)/F32</f>
         <v>1</v>
       </c>
     </row>
     <row r="33" spans="2:8">
-      <c r="B33" s="21" t="s">
+      <c r="B33" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="C33" s="21">
+      <c r="C33" s="23">
         <v>0</v>
       </c>
-      <c r="D33" s="21">
+      <c r="D33" s="23">
         <v>20</v>
       </c>
-      <c r="E33" s="21" t="s">
+      <c r="E33" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="F33" s="21">
+      <c r="F33" s="23">
         <v>45</v>
       </c>
-      <c r="G33" s="21">
+      <c r="G33" s="23">
         <v>0</v>
       </c>
-      <c r="H33" s="21">
+      <c r="H33" s="23">
         <f t="shared" si="7"/>
         <v>1</v>
       </c>
     </row>
     <row r="34" spans="2:8">
-      <c r="B34" s="21" t="s">
+      <c r="B34" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="C34" s="21">
+      <c r="C34" s="23">
         <v>0</v>
       </c>
-      <c r="D34" s="21">
+      <c r="D34" s="23">
         <v>20</v>
       </c>
-      <c r="E34" s="21" t="s">
+      <c r="E34" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="F34" s="21">
+      <c r="F34" s="23">
         <v>45</v>
       </c>
-      <c r="G34" s="21">
+      <c r="G34" s="23">
         <v>0</v>
       </c>
-      <c r="H34" s="21">
+      <c r="H34" s="23">
         <f t="shared" si="7"/>
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="2:8">
-      <c r="B35" s="21" t="s">
+      <c r="B35" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="C35" s="21">
+      <c r="C35" s="23">
         <v>0</v>
       </c>
-      <c r="D35" s="21">
+      <c r="D35" s="23">
         <v>20</v>
       </c>
-      <c r="E35" s="21" t="s">
+      <c r="E35" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="F35" s="21">
+      <c r="F35" s="23">
         <v>45</v>
       </c>
-      <c r="G35" s="21">
+      <c r="G35" s="23">
         <v>0</v>
       </c>
-      <c r="H35" s="21">
+      <c r="H35" s="23">
         <f t="shared" si="7"/>
         <v>1</v>
       </c>
     </row>
     <row r="36" spans="2:8">
-      <c r="B36" s="21" t="s">
+      <c r="B36" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="C36" s="21">
+      <c r="C36" s="23">
         <v>0</v>
       </c>
-      <c r="D36" s="21">
+      <c r="D36" s="23">
         <v>40</v>
       </c>
-      <c r="E36" s="21" t="s">
+      <c r="E36" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="F36" s="21">
+      <c r="F36" s="23">
         <v>45</v>
       </c>
-      <c r="G36" s="21">
+      <c r="G36" s="23">
         <v>0</v>
       </c>
-      <c r="H36" s="21">
+      <c r="H36" s="23">
         <f t="shared" si="7"/>
         <v>1</v>
       </c>
     </row>
     <row r="37" spans="2:8">
-      <c r="B37" s="21" t="s">
+      <c r="B37" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="C37" s="21">
+      <c r="C37" s="23">
         <v>0</v>
       </c>
-      <c r="D37" s="21">
+      <c r="D37" s="23">
         <v>60</v>
       </c>
-      <c r="E37" s="21" t="s">
+      <c r="E37" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="F37" s="21">
+      <c r="F37" s="23">
         <v>45</v>
       </c>
-      <c r="G37" s="21">
+      <c r="G37" s="23">
         <v>0</v>
       </c>
-      <c r="H37" s="21">
+      <c r="H37" s="23">
         <f t="shared" si="7"/>
         <v>1</v>
       </c>
     </row>
     <row r="38" spans="2:8">
-      <c r="B38" s="21" t="s">
+      <c r="B38" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="C38" s="21">
+      <c r="C38" s="23">
         <v>0</v>
       </c>
-      <c r="D38" s="21">
+      <c r="D38" s="23">
         <v>80</v>
       </c>
-      <c r="E38" s="21" t="s">
+      <c r="E38" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="F38" s="21">
+      <c r="F38" s="23">
         <v>45</v>
       </c>
-      <c r="G38" s="21">
+      <c r="G38" s="23">
         <v>0</v>
       </c>
-      <c r="H38" s="21">
+      <c r="H38" s="23">
         <f t="shared" si="7"/>
         <v>1</v>
       </c>
     </row>
     <row r="39" spans="2:8">
-      <c r="B39" s="21" t="s">
+      <c r="B39" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="C39" s="21">
+      <c r="C39" s="23">
         <v>0</v>
       </c>
-      <c r="D39" s="21">
+      <c r="D39" s="23">
         <v>100</v>
       </c>
-      <c r="E39" s="21" t="s">
+      <c r="E39" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="F39" s="21">
+      <c r="F39" s="23">
         <v>45</v>
       </c>
-      <c r="G39" s="21">
+      <c r="G39" s="23">
         <v>0</v>
       </c>
-      <c r="H39" s="21">
+      <c r="H39" s="23">
         <f t="shared" si="7"/>
         <v>1</v>
       </c>
     </row>
     <row r="40" spans="2:8">
-      <c r="B40" s="21" t="s">
+      <c r="B40" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="C40" s="21">
+      <c r="C40" s="23">
         <v>0</v>
       </c>
-      <c r="D40" s="21">
+      <c r="D40" s="23">
         <v>100</v>
       </c>
-      <c r="E40" s="21" t="s">
+      <c r="E40" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="F40" s="21">
+      <c r="F40" s="23">
         <v>45</v>
       </c>
-      <c r="G40" s="21">
+      <c r="G40" s="23">
         <v>15</v>
       </c>
-      <c r="H40" s="21">
+      <c r="H40" s="23">
         <f t="shared" si="7"/>
         <v>0.666666666666667</v>
       </c>
     </row>
     <row r="41" spans="2:8">
-      <c r="B41" s="21"/>
-      <c r="C41" s="21"/>
-      <c r="D41" s="21"/>
-      <c r="E41" s="21"/>
-      <c r="F41" s="21"/>
-      <c r="G41" s="21"/>
-      <c r="H41" s="21"/>
+      <c r="B41" s="23"/>
+      <c r="C41" s="23"/>
+      <c r="D41" s="23"/>
+      <c r="E41" s="23"/>
+      <c r="F41" s="23"/>
+      <c r="G41" s="23"/>
+      <c r="H41" s="23"/>
     </row>
     <row r="42" spans="2:8">
-      <c r="B42" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="C42" s="21">
-        <v>1</v>
-      </c>
-      <c r="D42" s="21">
+      <c r="B42" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="C42" s="23">
+        <v>1</v>
+      </c>
+      <c r="D42" s="23">
         <v>100</v>
       </c>
-      <c r="E42" s="21" t="s">
+      <c r="E42" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="F42" s="21">
+      <c r="F42" s="23">
         <v>75</v>
       </c>
-      <c r="G42" s="21">
+      <c r="G42" s="23">
         <v>30</v>
       </c>
-      <c r="H42" s="21">
+      <c r="H42" s="23">
         <f t="shared" ref="H42:H45" si="8">(F42-G42)/F42</f>
         <v>0.6</v>
       </c>
     </row>
     <row r="43" spans="2:8">
-      <c r="B43" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="C43" s="21">
+      <c r="B43" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="C43" s="23">
         <f t="shared" ref="C43:C45" si="9">D43*0.5</f>
         <v>200</v>
       </c>
-      <c r="D43" s="21">
+      <c r="D43" s="23">
         <v>400</v>
       </c>
-      <c r="E43" s="21" t="s">
+      <c r="E43" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="F43" s="21">
+      <c r="F43" s="23">
         <v>75</v>
       </c>
-      <c r="G43" s="21">
+      <c r="G43" s="23">
         <v>45</v>
       </c>
-      <c r="H43" s="21">
+      <c r="H43" s="23">
         <f t="shared" si="8"/>
         <v>0.4</v>
       </c>
     </row>
     <row r="44" spans="2:8">
-      <c r="B44" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="C44" s="21">
+      <c r="B44" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C44" s="23">
         <f t="shared" si="9"/>
         <v>400</v>
       </c>
-      <c r="D44" s="21">
+      <c r="D44" s="23">
         <v>800</v>
       </c>
-      <c r="E44" s="21" t="s">
+      <c r="E44" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="F44" s="21">
+      <c r="F44" s="23">
         <v>75</v>
       </c>
-      <c r="G44" s="21">
+      <c r="G44" s="23">
         <v>60</v>
       </c>
-      <c r="H44" s="21">
+      <c r="H44" s="23">
         <f t="shared" si="8"/>
         <v>0.2</v>
       </c>
     </row>
     <row r="45" spans="2:8">
-      <c r="B45" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="C45" s="21">
+      <c r="B45" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="C45" s="23">
         <f t="shared" si="9"/>
         <v>600</v>
       </c>
-      <c r="D45" s="21">
+      <c r="D45" s="23">
         <v>1200</v>
       </c>
-      <c r="E45" s="21" t="s">
+      <c r="E45" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="F45" s="21">
+      <c r="F45" s="23">
         <v>75</v>
       </c>
-      <c r="G45" s="21">
+      <c r="G45" s="23">
         <v>75</v>
       </c>
-      <c r="H45" s="21">
+      <c r="H45" s="23">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="46" spans="2:8">
-      <c r="B46" s="21"/>
-      <c r="C46" s="21"/>
-      <c r="D46" s="21"/>
-      <c r="E46" s="21"/>
-      <c r="F46" s="21"/>
-      <c r="G46" s="21"/>
-      <c r="H46" s="21"/>
+      <c r="B46" s="23"/>
+      <c r="C46" s="23"/>
+      <c r="D46" s="23"/>
+      <c r="E46" s="23"/>
+      <c r="F46" s="23"/>
+      <c r="G46" s="23"/>
+      <c r="H46" s="23"/>
     </row>
     <row r="47" spans="2:8">
-      <c r="B47" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="C47" s="21">
+      <c r="B47" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="C47" s="23">
         <f t="shared" ref="C47:C49" si="10">D47*0.5</f>
         <v>800</v>
       </c>
-      <c r="D47" s="21">
+      <c r="D47" s="23">
         <v>1600</v>
       </c>
-      <c r="E47" s="21" t="s">
+      <c r="E47" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="F47" s="21">
+      <c r="F47" s="23">
         <v>105</v>
       </c>
-      <c r="G47" s="21">
+      <c r="G47" s="23">
         <v>90</v>
       </c>
-      <c r="H47" s="21">
+      <c r="H47" s="23">
         <f t="shared" ref="H47:H49" si="11">(F47-G47)/F47</f>
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="48" spans="2:8">
-      <c r="B48" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="C48" s="21">
+      <c r="B48" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="C48" s="23">
         <f t="shared" si="10"/>
         <v>1000</v>
       </c>
-      <c r="D48" s="21">
+      <c r="D48" s="23">
         <v>2000</v>
       </c>
-      <c r="E48" s="21" t="s">
+      <c r="E48" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="F48" s="21">
+      <c r="F48" s="23">
         <v>105</v>
       </c>
-      <c r="G48" s="21">
+      <c r="G48" s="23">
         <v>105</v>
       </c>
-      <c r="H48" s="21">
+      <c r="H48" s="23">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
     </row>
     <row r="49" spans="2:8">
-      <c r="B49" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="C49" s="21">
+      <c r="B49" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="C49" s="23">
         <f t="shared" si="10"/>
         <v>1200</v>
       </c>
-      <c r="D49" s="21">
+      <c r="D49" s="23">
         <v>2400</v>
       </c>
-      <c r="E49" s="21" t="s">
+      <c r="E49" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="F49" s="21">
+      <c r="F49" s="23">
         <v>105</v>
       </c>
-      <c r="G49" s="21">
+      <c r="G49" s="23">
         <v>120</v>
       </c>
-      <c r="H49" s="21">
+      <c r="H49" s="23">
         <f t="shared" si="11"/>
         <v>-0.142857142857143</v>
       </c>
     </row>
     <row r="50" spans="2:8">
-      <c r="B50" s="21"/>
-      <c r="C50" s="21"/>
-      <c r="D50" s="21"/>
-      <c r="E50" s="21"/>
-      <c r="F50" s="21"/>
-      <c r="G50" s="21"/>
-      <c r="H50" s="21"/>
+      <c r="B50" s="23"/>
+      <c r="C50" s="23"/>
+      <c r="D50" s="23"/>
+      <c r="E50" s="23"/>
+      <c r="F50" s="23"/>
+      <c r="G50" s="23"/>
+      <c r="H50" s="23"/>
     </row>
     <row r="51" spans="2:8">
-      <c r="B51" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="C51" s="21">
+      <c r="B51" s="23" t="s">
+        <v>57</v>
+      </c>
+      <c r="C51" s="23">
         <f t="shared" ref="C51:C54" si="12">D51*0.5</f>
         <v>1400</v>
       </c>
-      <c r="D51" s="21">
+      <c r="D51" s="23">
         <v>2800</v>
       </c>
-      <c r="E51" s="21" t="s">
+      <c r="E51" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="F51" s="21">
+      <c r="F51" s="23">
         <v>135</v>
       </c>
-      <c r="G51" s="21">
+      <c r="G51" s="23">
         <v>135</v>
       </c>
-      <c r="H51" s="21">
+      <c r="H51" s="23">
         <f t="shared" ref="H51:H54" si="13">(F51-G51)/F51</f>
         <v>0</v>
       </c>
     </row>
     <row r="52" spans="2:8">
-      <c r="B52" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="C52" s="21">
+      <c r="B52" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="C52" s="23">
         <f t="shared" si="12"/>
         <v>1600</v>
       </c>
-      <c r="D52" s="21">
+      <c r="D52" s="23">
         <v>3200</v>
       </c>
-      <c r="E52" s="21" t="s">
+      <c r="E52" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="F52" s="21">
+      <c r="F52" s="23">
         <v>135</v>
       </c>
-      <c r="G52" s="21">
+      <c r="G52" s="23">
         <v>150</v>
       </c>
-      <c r="H52" s="21">
+      <c r="H52" s="23">
         <f t="shared" si="13"/>
         <v>-0.111111111111111</v>
       </c>
     </row>
     <row r="53" spans="2:8">
-      <c r="B53" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="C53" s="21">
+      <c r="B53" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C53" s="23">
         <f t="shared" si="12"/>
         <v>1800</v>
       </c>
-      <c r="D53" s="21">
+      <c r="D53" s="23">
         <v>3600</v>
       </c>
-      <c r="E53" s="21" t="s">
+      <c r="E53" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="F53" s="21">
+      <c r="F53" s="23">
         <v>135</v>
       </c>
-      <c r="G53" s="21">
+      <c r="G53" s="23">
         <v>175</v>
       </c>
-      <c r="H53" s="21">
+      <c r="H53" s="23">
         <f t="shared" si="13"/>
         <v>-0.296296296296296</v>
       </c>
     </row>
     <row r="54" spans="2:8">
-      <c r="B54" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="C54" s="21">
+      <c r="B54" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="C54" s="23">
         <f t="shared" si="12"/>
         <v>2000</v>
       </c>
-      <c r="D54" s="21">
+      <c r="D54" s="23">
         <v>4000</v>
       </c>
-      <c r="E54" s="21" t="s">
+      <c r="E54" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="F54" s="21">
+      <c r="F54" s="23">
         <v>135</v>
       </c>
-      <c r="G54" s="21">
+      <c r="G54" s="23">
         <v>190</v>
       </c>
-      <c r="H54" s="21">
+      <c r="H54" s="23">
         <f t="shared" si="13"/>
         <v>-0.407407407407407</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="34">
     <mergeCell ref="K2:O2"/>
     <mergeCell ref="P2:W2"/>
     <mergeCell ref="K3:O3"/>
@@ -3298,6 +3390,7 @@
     <mergeCell ref="L22:M22"/>
     <mergeCell ref="J23:K23"/>
     <mergeCell ref="L23:M23"/>
+    <mergeCell ref="C27:H27"/>
     <mergeCell ref="B30:H30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3313,549 +3406,552 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" customHeight="1"/>
   <cols>
     <col min="4" max="4" width="7.5" customWidth="1"/>
-    <col min="5" max="5" width="4.5" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="14.375" customWidth="1"/>
-    <col min="7" max="7" width="5.375" customWidth="1"/>
+    <col min="5" max="5" width="0.5" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="7" width="4.5" customWidth="1"/>
     <col min="9" max="9" width="4.5" customWidth="1"/>
-    <col min="10" max="10" width="4.25" customWidth="1"/>
+    <col min="10" max="10" width="3.125" customWidth="1"/>
     <col min="11" max="11" width="11.5" customWidth="1"/>
-    <col min="12" max="12" width="4.125" customWidth="1"/>
+    <col min="12" max="12" width="2.875" customWidth="1"/>
     <col min="13" max="13" width="10.5" customWidth="1"/>
-    <col min="14" max="14" width="4.625" customWidth="1"/>
-    <col min="15" max="15" width="18.875" style="1" customWidth="1"/>
-    <col min="16" max="16" width="4.125" customWidth="1"/>
-    <col min="17" max="17" width="19.25" customWidth="1"/>
+    <col min="14" max="14" width="3" customWidth="1"/>
+    <col min="15" max="15" width="17.625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="2.625" customWidth="1"/>
+    <col min="17" max="17" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="6" customHeight="1" spans="6:17">
       <c r="F6" s="2" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="O6" s="3"/>
-      <c r="P6" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="Q6" s="3"/>
+      <c r="H6" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="I6" s="4"/>
+      <c r="J6" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="O6" s="5"/>
+      <c r="P6" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q6" s="5"/>
     </row>
     <row r="7" customHeight="1" spans="6:17">
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G7" s="5">
-        <v>1</v>
-      </c>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5">
+      <c r="G7" s="7">
+        <v>1</v>
+      </c>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7">
         <v>0.8</v>
       </c>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5">
+      <c r="L7" s="7"/>
+      <c r="M7" s="7">
         <v>0.2</v>
       </c>
-      <c r="N7" s="5"/>
-      <c r="O7" s="6">
+      <c r="N7" s="7"/>
+      <c r="O7" s="8">
         <v>-0.3</v>
       </c>
-      <c r="P7" s="5"/>
-      <c r="Q7" s="7">
+      <c r="P7" s="7"/>
+      <c r="Q7" s="9">
         <v>-0.7</v>
       </c>
     </row>
     <row r="8" customHeight="1" spans="6:17">
-      <c r="F8" s="8">
+      <c r="F8" s="10">
         <v>30</v>
       </c>
-      <c r="G8" s="8"/>
-      <c r="H8" s="9" t="s">
+      <c r="G8" s="10"/>
+      <c r="H8" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9">
-        <v>1</v>
-      </c>
-      <c r="K8" s="9">
+      <c r="I8" s="11"/>
+      <c r="J8" s="11">
+        <v>1</v>
+      </c>
+      <c r="K8" s="11">
         <f ca="1" t="shared" ref="K8:K11" si="0">F8*K$9</f>
         <v>24</v>
       </c>
-      <c r="L8" s="9">
+      <c r="L8" s="11">
         <v>2</v>
       </c>
-      <c r="M8" s="9">
+      <c r="M8" s="11">
         <f ca="1" t="shared" ref="M8:M11" si="1">F8*M$9</f>
         <v>6</v>
       </c>
-      <c r="N8" s="9">
+      <c r="N8" s="11">
         <v>3</v>
       </c>
-      <c r="O8" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="P8" s="9">
+      <c r="O8" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="P8" s="11">
         <v>4</v>
       </c>
-      <c r="Q8" s="11" t="s">
-        <v>65</v>
+      <c r="Q8" s="13" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="9" customHeight="1" spans="6:17">
-      <c r="F9" s="4">
+      <c r="F9" s="6">
         <v>55</v>
       </c>
-      <c r="G9" s="4"/>
-      <c r="H9" s="5" t="s">
+      <c r="G9" s="6"/>
+      <c r="H9" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5">
-        <v>1</v>
-      </c>
-      <c r="K9" s="5">
+      <c r="I9" s="7"/>
+      <c r="J9" s="7">
+        <v>1</v>
+      </c>
+      <c r="K9" s="7">
         <f ca="1" t="shared" si="0"/>
         <v>44</v>
       </c>
-      <c r="L9" s="5">
+      <c r="L9" s="7">
         <v>2</v>
       </c>
-      <c r="M9" s="5">
+      <c r="M9" s="7">
         <f ca="1" t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="N9" s="5">
+      <c r="N9" s="7">
         <v>3</v>
       </c>
-      <c r="O9" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="P9" s="5">
+      <c r="O9" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="P9" s="7">
         <v>4</v>
       </c>
-      <c r="Q9" s="12" t="s">
-        <v>65</v>
+      <c r="Q9" s="14" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="10" customHeight="1" spans="6:17">
-      <c r="F10" s="8">
+      <c r="F10" s="10">
         <v>95</v>
       </c>
-      <c r="G10" s="8"/>
-      <c r="H10" s="9" t="s">
+      <c r="G10" s="10"/>
+      <c r="H10" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9">
-        <v>1</v>
-      </c>
-      <c r="K10" s="9">
+      <c r="I10" s="11"/>
+      <c r="J10" s="11">
+        <v>1</v>
+      </c>
+      <c r="K10" s="11">
         <f ca="1" t="shared" si="0"/>
         <v>76</v>
       </c>
-      <c r="L10" s="9">
+      <c r="L10" s="11">
         <v>2</v>
       </c>
-      <c r="M10" s="9">
+      <c r="M10" s="11">
         <f ca="1" t="shared" si="1"/>
         <v>19</v>
       </c>
-      <c r="N10" s="9">
+      <c r="N10" s="11">
         <v>3</v>
       </c>
-      <c r="O10" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="P10" s="9">
+      <c r="O10" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="P10" s="11">
         <v>4</v>
       </c>
-      <c r="Q10" s="11" t="s">
-        <v>65</v>
+      <c r="Q10" s="13" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="11" customHeight="1" spans="6:17">
-      <c r="F11" s="4">
+      <c r="F11" s="6">
         <v>135</v>
       </c>
-      <c r="G11" s="4"/>
-      <c r="H11" s="5" t="s">
+      <c r="G11" s="6"/>
+      <c r="H11" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5">
-        <v>1</v>
-      </c>
-      <c r="K11" s="5">
+      <c r="I11" s="7"/>
+      <c r="J11" s="7">
+        <v>1</v>
+      </c>
+      <c r="K11" s="7">
         <f ca="1" t="shared" si="0"/>
         <v>108</v>
       </c>
-      <c r="L11" s="5">
+      <c r="L11" s="7">
         <v>2</v>
       </c>
-      <c r="M11" s="5">
+      <c r="M11" s="7">
         <f ca="1" t="shared" si="1"/>
         <v>27</v>
       </c>
-      <c r="N11" s="5">
+      <c r="N11" s="7">
         <v>3</v>
       </c>
-      <c r="O11" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="P11" s="5">
+      <c r="O11" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="P11" s="7">
         <v>4</v>
       </c>
-      <c r="Q11" s="12" t="s">
-        <v>65</v>
+      <c r="Q11" s="14" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="12" customHeight="1" spans="6:17">
-      <c r="F12" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="G12" s="9">
+      <c r="F12" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="G12" s="11">
         <v>0.7</v>
       </c>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="9"/>
-      <c r="N12" s="9"/>
-      <c r="O12" s="10"/>
-      <c r="P12" s="9"/>
-      <c r="Q12" s="13"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="11"/>
+      <c r="N12" s="11"/>
+      <c r="O12" s="12"/>
+      <c r="P12" s="11"/>
+      <c r="Q12" s="15"/>
     </row>
     <row r="13" customHeight="1" spans="6:17">
-      <c r="F13" s="4">
+      <c r="F13" s="6">
         <f>F8*G$12</f>
         <v>21</v>
       </c>
-      <c r="G13" s="4"/>
-      <c r="H13" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5">
-        <v>1</v>
-      </c>
-      <c r="K13" s="5">
+      <c r="G13" s="6"/>
+      <c r="H13" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7">
+        <v>1</v>
+      </c>
+      <c r="K13" s="7">
         <f ca="1" t="shared" ref="K13:K16" si="2">F13*K$9</f>
         <v>16.8</v>
       </c>
-      <c r="L13" s="5">
+      <c r="L13" s="7">
         <v>2</v>
       </c>
-      <c r="M13" s="5">
+      <c r="M13" s="7">
         <f ca="1" t="shared" ref="M13:M16" si="3">F13*M$9</f>
         <v>4.2</v>
       </c>
-      <c r="N13" s="5">
+      <c r="N13" s="7">
         <v>3</v>
       </c>
-      <c r="O13" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="P13" s="5">
+      <c r="O13" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="P13" s="7">
         <v>4</v>
       </c>
-      <c r="Q13" s="12" t="s">
-        <v>67</v>
+      <c r="Q13" s="14" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="14" customHeight="1" spans="6:17">
-      <c r="F14" s="8">
+      <c r="F14" s="10">
         <f>F9*G$12</f>
         <v>38.5</v>
       </c>
-      <c r="G14" s="8"/>
-      <c r="H14" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9">
-        <v>1</v>
-      </c>
-      <c r="K14" s="9">
+      <c r="G14" s="10"/>
+      <c r="H14" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11">
+        <v>1</v>
+      </c>
+      <c r="K14" s="11">
         <f ca="1" t="shared" si="2"/>
         <v>30.8</v>
       </c>
-      <c r="L14" s="9">
+      <c r="L14" s="11">
         <v>2</v>
       </c>
-      <c r="M14" s="9">
+      <c r="M14" s="11">
         <f ca="1" t="shared" si="3"/>
         <v>7.7</v>
       </c>
-      <c r="N14" s="9">
+      <c r="N14" s="11">
         <v>3</v>
       </c>
-      <c r="O14" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="P14" s="9">
+      <c r="O14" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="P14" s="11">
         <v>4</v>
       </c>
-      <c r="Q14" s="11" t="s">
-        <v>67</v>
+      <c r="Q14" s="13" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="15" customHeight="1" spans="6:17">
-      <c r="F15" s="4">
+      <c r="F15" s="6">
         <f>F10*G$12</f>
         <v>66.5</v>
       </c>
-      <c r="G15" s="4"/>
-      <c r="H15" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5">
-        <v>1</v>
-      </c>
-      <c r="K15" s="5">
+      <c r="G15" s="6"/>
+      <c r="H15" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7">
+        <v>1</v>
+      </c>
+      <c r="K15" s="7">
         <f ca="1" t="shared" si="2"/>
         <v>53.2</v>
       </c>
-      <c r="L15" s="5">
+      <c r="L15" s="7">
         <v>2</v>
       </c>
-      <c r="M15" s="5">
+      <c r="M15" s="7">
         <f ca="1" t="shared" si="3"/>
         <v>13.3</v>
       </c>
-      <c r="N15" s="5">
+      <c r="N15" s="7">
         <v>3</v>
       </c>
-      <c r="O15" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="P15" s="5">
+      <c r="O15" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="P15" s="7">
         <v>4</v>
       </c>
-      <c r="Q15" s="12" t="s">
-        <v>67</v>
+      <c r="Q15" s="14" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="16" customHeight="1" spans="6:17">
-      <c r="F16" s="8">
+      <c r="F16" s="10">
         <f>F11*G$12</f>
         <v>94.5</v>
       </c>
-      <c r="G16" s="8"/>
-      <c r="H16" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9">
-        <v>1</v>
-      </c>
-      <c r="K16" s="9">
+      <c r="G16" s="10"/>
+      <c r="H16" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11">
+        <v>1</v>
+      </c>
+      <c r="K16" s="11">
         <f ca="1" t="shared" si="2"/>
         <v>75.6</v>
       </c>
-      <c r="L16" s="9">
+      <c r="L16" s="11">
         <v>2</v>
       </c>
-      <c r="M16" s="9">
+      <c r="M16" s="11">
         <f ca="1" t="shared" si="3"/>
         <v>18.9</v>
       </c>
-      <c r="N16" s="9">
+      <c r="N16" s="11">
         <v>3</v>
       </c>
-      <c r="O16" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="P16" s="9">
+      <c r="O16" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="P16" s="11">
         <v>4</v>
       </c>
-      <c r="Q16" s="11" t="s">
-        <v>67</v>
+      <c r="Q16" s="13" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="17" customHeight="1" spans="6:17">
-      <c r="F17" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="G17" s="5">
+      <c r="F17" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="G17" s="7">
         <v>0.49</v>
       </c>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-      <c r="N17" s="5"/>
-      <c r="O17" s="6"/>
-      <c r="P17" s="5"/>
-      <c r="Q17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="8"/>
+      <c r="P17" s="7"/>
+      <c r="Q17" s="9"/>
     </row>
     <row r="18" customHeight="1" spans="6:17">
-      <c r="F18" s="8">
+      <c r="F18" s="10">
         <f>F8*G$17</f>
         <v>14.7</v>
       </c>
-      <c r="G18" s="8"/>
-      <c r="H18" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9">
-        <v>1</v>
-      </c>
-      <c r="K18" s="9">
+      <c r="G18" s="10"/>
+      <c r="H18" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11">
+        <v>1</v>
+      </c>
+      <c r="K18" s="11">
         <f ca="1" t="shared" ref="K18:K21" si="4">F18*K$9</f>
         <v>11.76</v>
       </c>
-      <c r="L18" s="9">
+      <c r="L18" s="11">
         <v>2</v>
       </c>
-      <c r="M18" s="9">
+      <c r="M18" s="11">
         <f ca="1" t="shared" ref="M18:M21" si="5">F18*M$9</f>
         <v>2.94</v>
       </c>
-      <c r="N18" s="9">
+      <c r="N18" s="11">
         <v>3</v>
       </c>
-      <c r="O18" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="P18" s="9">
+      <c r="O18" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="P18" s="11">
         <v>4</v>
       </c>
-      <c r="Q18" s="11" t="s">
-        <v>69</v>
+      <c r="Q18" s="13" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="19" customHeight="1" spans="6:17">
-      <c r="F19" s="4">
+      <c r="F19" s="6">
         <f>F9*G$17</f>
         <v>26.95</v>
       </c>
-      <c r="G19" s="4"/>
-      <c r="H19" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5">
-        <v>1</v>
-      </c>
-      <c r="K19" s="5">
+      <c r="G19" s="6"/>
+      <c r="H19" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="I19" s="7"/>
+      <c r="J19" s="7">
+        <v>1</v>
+      </c>
+      <c r="K19" s="7">
         <f ca="1" t="shared" si="4"/>
         <v>21.56</v>
       </c>
-      <c r="L19" s="5">
+      <c r="L19" s="7">
         <v>2</v>
       </c>
-      <c r="M19" s="5">
+      <c r="M19" s="7">
         <f ca="1" t="shared" si="5"/>
         <v>5.39</v>
       </c>
-      <c r="N19" s="5">
+      <c r="N19" s="7">
         <v>3</v>
       </c>
-      <c r="O19" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="P19" s="5">
+      <c r="O19" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="P19" s="7">
         <v>4</v>
       </c>
-      <c r="Q19" s="12" t="s">
-        <v>69</v>
+      <c r="Q19" s="14" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="20" customHeight="1" spans="6:17">
-      <c r="F20" s="8">
+      <c r="F20" s="10">
         <f>F10*G$17</f>
         <v>46.55</v>
       </c>
-      <c r="G20" s="8"/>
-      <c r="H20" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9">
-        <v>1</v>
-      </c>
-      <c r="K20" s="9">
+      <c r="G20" s="10"/>
+      <c r="H20" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11">
+        <v>1</v>
+      </c>
+      <c r="K20" s="11">
         <f ca="1" t="shared" si="4"/>
         <v>37.24</v>
       </c>
-      <c r="L20" s="9">
+      <c r="L20" s="11">
         <v>2</v>
       </c>
-      <c r="M20" s="9">
+      <c r="M20" s="11">
         <f ca="1" t="shared" si="5"/>
         <v>9.31</v>
       </c>
-      <c r="N20" s="9">
+      <c r="N20" s="11">
         <v>3</v>
       </c>
-      <c r="O20" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="P20" s="9">
+      <c r="O20" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="P20" s="11">
         <v>4</v>
       </c>
-      <c r="Q20" s="11" t="s">
-        <v>69</v>
+      <c r="Q20" s="13" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="21" customHeight="1" spans="6:17">
-      <c r="F21" s="14">
+      <c r="F21" s="16">
         <f>F11*G$17</f>
         <v>66.15</v>
       </c>
-      <c r="G21" s="14"/>
-      <c r="H21" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="I21" s="15"/>
-      <c r="J21" s="15">
-        <v>1</v>
-      </c>
-      <c r="K21" s="15">
+      <c r="G21" s="16"/>
+      <c r="H21" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="I21" s="17"/>
+      <c r="J21" s="17">
+        <v>1</v>
+      </c>
+      <c r="K21" s="17">
         <f ca="1" t="shared" si="4"/>
         <v>52.92</v>
       </c>
-      <c r="L21" s="15">
+      <c r="L21" s="17">
         <v>2</v>
       </c>
-      <c r="M21" s="15">
+      <c r="M21" s="17">
         <f ca="1" t="shared" si="5"/>
         <v>13.23</v>
       </c>
-      <c r="N21" s="15">
+      <c r="N21" s="17">
         <v>3</v>
       </c>
-      <c r="O21" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="P21" s="15">
+      <c r="O21" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="P21" s="17">
         <v>4</v>
       </c>
-      <c r="Q21" s="17" t="s">
-        <v>69</v>
+      <c r="Q21" s="19" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="30">
     <mergeCell ref="F6:G6"/>
+    <mergeCell ref="H6:I6"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="L6:M6"/>
     <mergeCell ref="N6:O6"/>

</xml_diff>